<commit_message>
fix(AJ15XIAOMI-9): sync updated frozen earphone list
更新EAR001-EAR008冻结产品名单
同步PROJECT_SCOPE中的产品范围和变更记录
</commit_message>
<xml_diff>
--- a/data/earphone_list.xlsx
+++ b/data/earphone_list.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="产品名单" sheetId="1" r:id="R0bf9844653f44999"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="选择说明" sheetId="2" r:id="R547816971f334d94"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="产品名单" sheetId="1" r:id="R7741b16a419540cc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="选择说明" sheetId="2" r:id="R78b2086f64a74609"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -51,7 +51,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="19">
+  <x:cellXfs count="20">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -89,6 +89,7 @@
     <x:xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -312,31 +313,31 @@
         <x:v>EAR001</x:v>
       </x:c>
       <x:c r="B2" s="12" t="str">
-        <x:v>REDMI Buds 8 青春版</x:v>
+        <x:v>小米真无线蓝牙耳机 Air2 SE</x:v>
       </x:c>
       <x:c r="C2" s="12" t="str">
-        <x:v>REDMI</x:v>
+        <x:v>Xiaomi</x:v>
       </x:c>
       <x:c r="D2" s="12" t="str">
         <x:v>入门</x:v>
       </x:c>
       <x:c r="E2" s="12" t="str">
-        <x:v>入耳式</x:v>
+        <x:v>半入耳式</x:v>
       </x:c>
       <x:c r="F2" s="12" t="str">
-        <x:v>https://www.mi.com/prod/redmi-buds-8-lite</x:v>
+        <x:v>https://www.mi.com/product/mi-true-wireless-earphone-2-se/</x:v>
       </x:c>
       <x:c r="G2" s="12" t="str">
-        <x:v>待核验</x:v>
+        <x:v>是</x:v>
       </x:c>
       <x:c r="H2" s="12" t="str">
-        <x:v>入门价位样本，适合预算敏感用户；与高端降噪产品形成明显差异</x:v>
+        <x:v>入门半入耳式样本，适合日常使用、轻便佩戴和基础续航对比</x:v>
       </x:c>
       <x:c r="I2" s="12" t="str">
-        <x:v>已确认官方产品页</x:v>
+        <x:v>已完成参数与说明书核验</x:v>
       </x:c>
       <x:c r="J2" s="12" t="str">
-        <x:v>具体型号与说明书由组员A核验</x:v>
+        <x:v>型号：TWSEJ04WM</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -344,31 +345,31 @@
         <x:v>EAR002</x:v>
       </x:c>
       <x:c r="B3" s="12" t="str">
-        <x:v>REDMI Buds 8 活力版</x:v>
+        <x:v>Xiaomi 真无线降噪耳机 3</x:v>
       </x:c>
       <x:c r="C3" s="12" t="str">
-        <x:v>REDMI</x:v>
+        <x:v>Xiaomi</x:v>
       </x:c>
       <x:c r="D3" s="12" t="str">
-        <x:v>入门</x:v>
+        <x:v>高端</x:v>
       </x:c>
       <x:c r="E3" s="12" t="str">
-        <x:v>半入耳式</x:v>
+        <x:v>入耳式</x:v>
       </x:c>
       <x:c r="F3" s="12" t="str">
-        <x:v>https://www.mi.com/prod/redmi-buds-8-active</x:v>
+        <x:v>https://www.mi.com/product/xiaomibuds3/</x:v>
       </x:c>
       <x:c r="G3" s="12" t="str">
-        <x:v>待核验</x:v>
+        <x:v>是</x:v>
       </x:c>
       <x:c r="H3" s="12" t="str">
-        <x:v>入门半入耳式样本，可用于轻便、舒适和日常场景推荐</x:v>
+        <x:v>高端主动降噪样本，适合降噪深度、续航和双设备功能对比</x:v>
       </x:c>
       <x:c r="I3" s="12" t="str">
-        <x:v>已确认官方产品页</x:v>
+        <x:v>已完成参数与说明书核验</x:v>
       </x:c>
       <x:c r="J3" s="12" t="str">
-        <x:v>说明书可用性待核验</x:v>
+        <x:v>型号：M2111E1</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -376,31 +377,31 @@
         <x:v>EAR003</x:v>
       </x:c>
       <x:c r="B4" s="12" t="str">
-        <x:v>REDMI Buds 7S</x:v>
+        <x:v>Redmi Buds 3 真无线蓝牙耳机</x:v>
       </x:c>
       <x:c r="C4" s="12" t="str">
         <x:v>REDMI</x:v>
       </x:c>
       <x:c r="D4" s="12" t="str">
-        <x:v>中端</x:v>
+        <x:v>入门</x:v>
       </x:c>
       <x:c r="E4" s="12" t="str">
         <x:v>半入耳式</x:v>
       </x:c>
       <x:c r="F4" s="12" t="str">
-        <x:v>https://www.mi.com/prod/redmi-buds-7s</x:v>
+        <x:v>https://www.mi.com/redmiPod/buds3/</x:v>
       </x:c>
       <x:c r="G4" s="12" t="str">
-        <x:v>待核验</x:v>
+        <x:v>是</x:v>
       </x:c>
       <x:c r="H4" s="12" t="str">
-        <x:v>中端半入耳式样本，用于对比佩戴方式、降噪和舒适性</x:v>
+        <x:v>入门半入耳式样本，适合佩戴舒适度、通话和低延迟功能对比</x:v>
       </x:c>
       <x:c r="I4" s="12" t="str">
-        <x:v>已确认官方产品页</x:v>
+        <x:v>已完成参数与说明书核验</x:v>
       </x:c>
       <x:c r="J4" s="12" t="str">
-        <x:v>详细功能参数待采集</x:v>
+        <x:v>型号：M2104E1</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -408,31 +409,31 @@
         <x:v>EAR004</x:v>
       </x:c>
       <x:c r="B5" s="12" t="str">
-        <x:v>REDMI Buds 8</x:v>
+        <x:v>Redmi Buds 3 青春版</x:v>
       </x:c>
       <x:c r="C5" s="12" t="str">
         <x:v>REDMI</x:v>
       </x:c>
       <x:c r="D5" s="12" t="str">
-        <x:v>中端</x:v>
+        <x:v>入门</x:v>
       </x:c>
       <x:c r="E5" s="12" t="str">
         <x:v>入耳式</x:v>
       </x:c>
       <x:c r="F5" s="12" t="str">
-        <x:v>https://www.mi.com/prod/redmi-buds-8</x:v>
+        <x:v>https://www.mi.com/product/redmi-buds-3-lite/</x:v>
       </x:c>
       <x:c r="G5" s="12" t="str">
-        <x:v>待核验</x:v>
+        <x:v>是</x:v>
       </x:c>
       <x:c r="H5" s="12" t="str">
-        <x:v>新一代中端降噪样本，适合通勤、续航和综合功能比较</x:v>
+        <x:v>低价入耳式样本，适合预算敏感、运动和游戏低延迟场景推荐</x:v>
       </x:c>
       <x:c r="I5" s="12" t="str">
-        <x:v>已确认官方产品页</x:v>
+        <x:v>已完成参数与说明书核验</x:v>
       </x:c>
       <x:c r="J5" s="12" t="str">
-        <x:v>详细价格和参数待采集</x:v>
+        <x:v>型号：M2110E1</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -440,31 +441,31 @@
         <x:v>EAR005</x:v>
       </x:c>
       <x:c r="B6" s="12" t="str">
-        <x:v>REDMI Buds 6</x:v>
+        <x:v>Xiaomi Buds 4</x:v>
       </x:c>
       <x:c r="C6" s="12" t="str">
-        <x:v>REDMI</x:v>
+        <x:v>Xiaomi</x:v>
       </x:c>
       <x:c r="D6" s="12" t="str">
-        <x:v>中端</x:v>
+        <x:v>高端</x:v>
       </x:c>
       <x:c r="E6" s="12" t="str">
-        <x:v>入耳式</x:v>
+        <x:v>半入耳式</x:v>
       </x:c>
       <x:c r="F6" s="12" t="str">
-        <x:v>https://www.mi.com/prod/redmi-buds-6</x:v>
+        <x:v>https://www.mi.com/xiaomi-buds-4/</x:v>
       </x:c>
       <x:c r="G6" s="12" t="str">
-        <x:v>待核验</x:v>
+        <x:v>是</x:v>
       </x:c>
       <x:c r="H6" s="12" t="str">
-        <x:v>成熟中端样本，官方支持资料较丰富，适合RAG问答验证</x:v>
+        <x:v>高端半入耳式主动降噪样本，适合音质、降噪和舒适性对比</x:v>
       </x:c>
       <x:c r="I6" s="12" t="str">
-        <x:v>已确认官方产品页</x:v>
+        <x:v>已完成参数与说明书核验</x:v>
       </x:c>
       <x:c r="J6" s="12" t="str">
-        <x:v>可优先查找官方FAQ或说明书</x:v>
+        <x:v>型号：M2224E1</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -472,31 +473,31 @@
         <x:v>EAR006</x:v>
       </x:c>
       <x:c r="B7" s="12" t="str">
-        <x:v>REDMI Buds 8 Pro</x:v>
+        <x:v>Redmi Buds 4 Pro</x:v>
       </x:c>
       <x:c r="C7" s="12" t="str">
         <x:v>REDMI</x:v>
       </x:c>
       <x:c r="D7" s="12" t="str">
-        <x:v>高端</x:v>
+        <x:v>中端</x:v>
       </x:c>
       <x:c r="E7" s="12" t="str">
         <x:v>入耳式</x:v>
       </x:c>
       <x:c r="F7" s="12" t="str">
-        <x:v>https://www.mi.com/prod/redmi-buds-8-pro</x:v>
+        <x:v>https://www.mi.com/redmibuds4pro/</x:v>
       </x:c>
       <x:c r="G7" s="12" t="str">
-        <x:v>待核验</x:v>
+        <x:v>是</x:v>
       </x:c>
       <x:c r="H7" s="12" t="str">
-        <x:v>高端主动降噪样本，用于降噪、音质和双设备功能对比</x:v>
+        <x:v>中端主动降噪样本，适合降噪、长续航、双设备和游戏场景推荐</x:v>
       </x:c>
       <x:c r="I7" s="12" t="str">
-        <x:v>已确认官方产品页</x:v>
+        <x:v>已完成参数与说明书核验</x:v>
       </x:c>
       <x:c r="J7" s="12" t="str">
-        <x:v>作为重点说明书候选</x:v>
+        <x:v>型号：M2132E1</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -504,31 +505,31 @@
         <x:v>EAR007</x:v>
       </x:c>
       <x:c r="B8" s="12" t="str">
-        <x:v>Xiaomi Buds 6</x:v>
+        <x:v>Redmi Buds 4 青春版</x:v>
       </x:c>
       <x:c r="C8" s="12" t="str">
-        <x:v>Xiaomi</x:v>
+        <x:v>REDMI</x:v>
       </x:c>
       <x:c r="D8" s="12" t="str">
-        <x:v>高端</x:v>
+        <x:v>入门</x:v>
       </x:c>
       <x:c r="E8" s="12" t="str">
-        <x:v>待核验</x:v>
+        <x:v>半入耳式</x:v>
       </x:c>
       <x:c r="F8" s="12" t="str">
-        <x:v>https://www.mi.com/prod/xiaomi-buds-6</x:v>
+        <x:v>https://www.mi.com/redmi-buds-4-lite/</x:v>
       </x:c>
       <x:c r="G8" s="12" t="str">
-        <x:v>待核验</x:v>
+        <x:v>是</x:v>
       </x:c>
       <x:c r="H8" s="12" t="str">
-        <x:v>Xiaomi旗舰产品样本，用于高端产品与REDMI产品线对比</x:v>
+        <x:v>入门轻量半入耳式样本，适合日常、轻便和低延迟场景推荐</x:v>
       </x:c>
       <x:c r="I8" s="12" t="str">
-        <x:v>已确认官方产品页</x:v>
+        <x:v>已完成参数与说明书核验</x:v>
       </x:c>
       <x:c r="J8" s="12" t="str">
-        <x:v>佩戴方式、型号和说明书待核验</x:v>
+        <x:v>型号：M2231E1</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -536,31 +537,31 @@
         <x:v>EAR008</x:v>
       </x:c>
       <x:c r="B9" s="12" t="str">
-        <x:v>Xiaomi 开放式耳机 Pro</x:v>
+        <x:v>Redmi Buds 4</x:v>
       </x:c>
       <x:c r="C9" s="12" t="str">
-        <x:v>Xiaomi</x:v>
+        <x:v>REDMI</x:v>
       </x:c>
       <x:c r="D9" s="12" t="str">
-        <x:v>开放式</x:v>
+        <x:v>中端</x:v>
       </x:c>
       <x:c r="E9" s="12" t="str">
-        <x:v>开放式</x:v>
+        <x:v>入耳式</x:v>
       </x:c>
       <x:c r="F9" s="12" t="str">
-        <x:v>https://www.mi.com/prod/xiaomi-open-earphones-pro</x:v>
+        <x:v>https://www.mi.com/redmibuds4/</x:v>
       </x:c>
       <x:c r="G9" s="12" t="str">
-        <x:v>待核验</x:v>
+        <x:v>是</x:v>
       </x:c>
       <x:c r="H9" s="12" t="str">
-        <x:v>开放式产品样本，用于不接受入耳式、长时间佩戴等需求推荐</x:v>
+        <x:v>中端主动降噪样本，适合通勤、续航、防水和低延迟功能对比</x:v>
       </x:c>
       <x:c r="I9" s="12" t="str">
-        <x:v>已确认官方产品页</x:v>
+        <x:v>已完成参数与说明书核验</x:v>
       </x:c>
       <x:c r="J9" s="12" t="str">
-        <x:v>作为特殊佩戴方式代表</x:v>
+        <x:v>型号：M2137E1</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -580,7 +581,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reb27817ff8b2449d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb5d521a005b3474f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -593,7 +594,7 @@
     <x:col min="2" max="2" width="80" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1">
+    <x:row r="1" ht="15" hidden="0" customHeight="1">
       <x:c r="A1" s="18" t="str">
         <x:v>项目</x:v>
       </x:c>
@@ -601,36 +602,44 @@
         <x:v>内容</x:v>
       </x:c>
     </x:row>
-    <x:row r="2">
+    <x:row r="2" ht="15" hidden="0" customHeight="1">
       <x:c r="A2" s="12" t="str">
         <x:v>选择原则</x:v>
       </x:c>
       <x:c r="B2" s="12" t="str">
-        <x:v>官方产品页可追溯、参数差异明显、覆盖多个价位和佩戴方式、至少4款可用于说明书问答</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3">
+        <x:v>官方产品页可追溯、参数差异明显、覆盖多个价位和佩戴方式、8款产品均可用于说明书问答</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="15" hidden="0" customHeight="1">
       <x:c r="A3" s="12" t="str">
         <x:v>产品结构</x:v>
       </x:c>
       <x:c r="B3" s="12" t="str">
-        <x:v>2款入门 + 3款中端 + 2款高端/旗舰 + 1款开放式</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4">
+        <x:v>4款入门 + 2款中端 + 2款高端；4款入耳式 + 4款半入耳式；本阶段不包含开放式产品</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="15" hidden="0" customHeight="1">
       <x:c r="A4" s="12" t="str">
         <x:v>当前状态</x:v>
       </x:c>
       <x:c r="B4" s="12" t="str">
-        <x:v>任务1仅冻结产品范围；具体型号、参数、价格和说明书可用性由任务2和任务3继续核验</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5">
+        <x:v>AJ15XIAOMI-10 产品数据与 AJ15XIAOMI-11 说明书资料已完成核验，当前名单作为第一阶段冻结范围</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="15" hidden="0" customHeight="1">
       <x:c r="A5" s="12" t="str">
         <x:v>变更规则</x:v>
       </x:c>
       <x:c r="B5" s="12" t="str">
-        <x:v>产品名单合并到main后，如需替换产品，必须在Jira记录原因并更新本表</x:v>
+        <x:v>产品名单合并到main后，如需再次替换产品，必须由组长确认，并在Jira及本表记录原因</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A6" t="str">
+        <x:v>变更记录</x:v>
+      </x:c>
+      <x:c r="B6" s="12" t="str">
+        <x:v>2026-07-17：经组长确认，冻结名单调整为当前8款产品，后续数据清洗、推荐算法和RAG均以EAR001—EAR008为准</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>